<commit_message>
documents the manual evaluation of the query analysis
</commit_message>
<xml_diff>
--- a/data/Prompt Evaluation.xlsx
+++ b/data/Prompt Evaluation.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/merlindconstanzepohl/Desktop/RAG Implementierung/Code/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B65A0CE0-10D5-9445-AED7-CA2AB318783C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B2FCE2-A494-7A4B-BC8F-E4B5A1E29FF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1040" yWindow="680" windowWidth="27620" windowHeight="16080" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="62">
   <si>
     <t>Query</t>
   </si>
@@ -176,30 +176,6 @@
 Do not say where the information comes from, just give the answer. 
 If the provided texts mention different numbers or information for the same topic, list them separately. 
     </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Context Recall</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Did the retriever find all the relevant information?
-Is all necessary information present in the retrieved chunks?</t>
     </r>
   </si>
   <si>
@@ -223,29 +199,6 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t>relevant (1)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-correct</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>partially relevant (1)</t>
     </r>
     <r>
@@ -261,6 +214,9 @@
     </r>
   </si>
   <si>
+    <t>Total reef visits increased from 1.4 million in 1993-94 to just under 2 million visits in 2004-05.(p. 23)</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -269,7 +225,7 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t>relevant</t>
+      <t>value provided in documents (1)</t>
     </r>
     <r>
       <rPr>
@@ -279,31 +235,74 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (1)
-correct</t>
-    </r>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>What does happen to the fish if the reef gets in a bad condition?</t>
+  </si>
+  <si>
+    <t>The fish and other organisms dependent on the living coral also die (if they cannot move elsewhere). In turn, the fish and other animals higher up the food chain (including the top predators) also either die or move elsewhere.</t>
+  </si>
+  <si>
+    <t>The text does not mention what happens to the octopus. It only discusses the effects of climate change on coral reefs and the organisms that depend on them, including fish and other animals higher up the food chain.</t>
+  </si>
+  <si>
+    <t>What happens to the octopus?</t>
+  </si>
+  <si>
+    <t>Where is Nemo?</t>
+  </si>
+  <si>
+    <t>There is no mention of Nemo in the provided context.</t>
+  </si>
+  <si>
+    <t>not int the document</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not in the document </t>
+  </si>
+  <si>
+    <t>Can we calculate the total population of Australia?</t>
+  </si>
+  <si>
+    <t>value provided in documents (1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value not provided in documents (1)
+</t>
+  </si>
+  <si>
+    <t>ECO-SYSTEM IMPACTS: The fish and other organisms dependent on the
+living coral also die (if they cannot move elsewhere). In turn, the fish and other animals
+higher up the food chain (including the top predators) also either die or move elsewhere. (p. 57/58)</t>
+  </si>
+  <si>
+    <t>No, the provided context does not mention the total population of Australia. It only provides information on the economic value and employment figures for the Great Barrier Reef Marine Park (GBRMP) in Queensland and Australia.</t>
   </si>
   <si>
     <r>
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">relevant (1) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>partially relevant (0)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-correct</t>
+it provides literally the same text, without the context before it seems a bit abstract and is not well readable
+</t>
     </r>
   </si>
   <si>
@@ -315,6 +314,30 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
+      <t>partially relevant (1)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+no hallucination/not wrong, still incorrect value because of wrong context -  but could be correct if user doesn't know
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>partially relevant (0)</t>
     </r>
     <r>
@@ -326,9 +349,53 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-no hallucination/not wrong, still value not correct because of wrong context
+no hallucination/not wrong, still value not correctly given and answer not properly answered
 </t>
     </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Correctness
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Retrieval output versus expected text/ground truth</t>
+    </r>
+  </si>
+  <si>
+    <t>not correct</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>relevant (1)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>correct</t>
   </si>
   <si>
     <r>
@@ -362,7 +429,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-Geht die Antwort  komplett an der Intention des Nutzers vorbei? Ist die antwort sinnvoll?</t>
+</t>
     </r>
   </si>
   <si>
@@ -388,95 +455,6 @@
 Does the answer come only from the provided documents? 
 Is the response supported by the context?
 Does the model hallucinate?
-Hält sich das modell an die regeln und gibt nur fakten aus dem text wieder?</t>
-    </r>
-  </si>
-  <si>
-    <t>Total reef visits increased from 1.4 million in 1993-94 to just under 2 million visits in 2004-05.(p. 23)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>value provided in documents (1)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <t>What does happen to the fish if the reef gets in a bad condition?</t>
-  </si>
-  <si>
-    <t>The fish and other organisms dependent on the living coral also die (if they cannot move elsewhere). In turn, the fish and other animals higher up the food chain (including the top predators) also either die or move elsewhere.</t>
-  </si>
-  <si>
-    <t>The text does not mention what happens to the octopus. It only discusses the effects of climate change on coral reefs and the organisms that depend on them, including fish and other animals higher up the food chain.</t>
-  </si>
-  <si>
-    <t>What happens to the octopus?</t>
-  </si>
-  <si>
-    <t>Where is Nemo?</t>
-  </si>
-  <si>
-    <t>There is no mention of Nemo in the provided context.</t>
-  </si>
-  <si>
-    <t>not int the document</t>
-  </si>
-  <si>
-    <t xml:space="preserve">not in the document </t>
-  </si>
-  <si>
-    <t>Can we calculate the total population of Australia?</t>
-  </si>
-  <si>
-    <t>value provided in documents (1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value not provided in documents (1)
-</t>
-  </si>
-  <si>
-    <t>ECO-SYSTEM IMPACTS: The fish and other organisms dependent on the
-living coral also die (if they cannot move elsewhere). In turn, the fish and other animals
-higher up the food chain (including the top predators) also either die or move elsewhere. (p. 57/58)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>partially relevant (1)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-no hallucination/not wrong, still value not correct because of wrong context but could be correct if user doesn't know
 </t>
     </r>
   </si>
@@ -554,7 +532,7 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Context Recall:</t>
+      <t>Correctness:</t>
     </r>
     <r>
       <rPr>
@@ -564,91 +542,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">
+      <t xml:space="preserve"> correct / not correct
 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>found all / found partially / not found</t>
-    </r>
-  </si>
-  <si>
-    <t>No, the provided context does not mention the total population of Australia. It only provides information on the economic value and employment figures for the Great Barrier Reef Marine Park (GBRMP) in Queensland and Australia.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>partially relevant (0)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-it provides literally the same text, without the context before it seems a bit abstract and is not well readable
-</t>
-    </r>
-  </si>
-  <si>
-    <t>not found (0)</t>
-  </si>
-  <si>
-    <t>found all (1)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>found partially (1)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-still a good answer and short, as LLM prompt instructed </t>
-    </r>
-  </si>
-  <si>
-    <t>not found (1)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">not found (0)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">in the same chunk there was the information about much the world will heat up (expected and estimated value), the answer was just not long enough. </t>
     </r>
   </si>
 </sst>
@@ -656,7 +551,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -674,26 +569,6 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
@@ -747,10 +622,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1092,17 +967,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{483B6C7E-3945-004D-9C20-B4D0D386A596}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="52.6640625" customWidth="1"/>
     <col min="3" max="4" width="42.1640625" customWidth="1"/>
     <col min="5" max="5" width="42.1640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="53.6640625" customWidth="1"/>
-    <col min="7" max="7" width="39.1640625" customWidth="1"/>
-    <col min="8" max="8" width="40.83203125" customWidth="1"/>
-    <col min="9" max="9" width="42" customWidth="1"/>
+    <col min="6" max="7" width="53.6640625" customWidth="1"/>
+    <col min="8" max="8" width="39.1640625" customWidth="1"/>
+    <col min="9" max="9" width="40.83203125" customWidth="1"/>
+    <col min="10" max="10" width="42" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="155" customHeight="1" x14ac:dyDescent="0.2">
@@ -1119,23 +994,23 @@
         <v>34</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>35</v>
+        <v>59</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="68" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="6" t="s">
@@ -1145,13 +1020,13 @@
         <v>19</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>62</v>
+        <v>53</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>56</v>
       </c>
       <c r="H2" s="1"/>
     </row>
@@ -1169,13 +1044,13 @@
         <v>20</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>63</v>
+        <v>57</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H3" s="1"/>
     </row>
@@ -1183,7 +1058,7 @@
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C4" s="6" t="s">
@@ -1193,13 +1068,13 @@
         <v>21</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>63</v>
+        <v>57</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H4" s="1"/>
     </row>
@@ -1207,7 +1082,7 @@
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -1217,13 +1092,13 @@
         <v>23</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>63</v>
+        <v>57</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H5" s="1"/>
     </row>
@@ -1231,23 +1106,23 @@
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>24</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>64</v>
+        <v>36</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H6" s="1"/>
     </row>
@@ -1265,13 +1140,13 @@
         <v>25</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>63</v>
+        <v>57</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H7" s="1"/>
     </row>
@@ -1279,7 +1154,7 @@
       <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="6" t="s">
@@ -1289,13 +1164,13 @@
         <v>26</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>63</v>
+        <v>57</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H8" s="1"/>
     </row>
@@ -1313,17 +1188,17 @@
         <v>27</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>63</v>
+        <v>57</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H9" s="1"/>
     </row>
-    <row r="10" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" ht="68" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1337,13 +1212,13 @@
         <v>28</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>66</v>
+        <v>54</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>56</v>
       </c>
       <c r="H10" s="1"/>
     </row>
@@ -1361,13 +1236,13 @@
         <v>29</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>63</v>
+        <v>38</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H11" s="1"/>
     </row>
@@ -1375,23 +1250,23 @@
       <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>10</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>30</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>63</v>
+        <v>57</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H12" s="1"/>
     </row>
@@ -1399,23 +1274,23 @@
       <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>46</v>
+      <c r="B13" s="8" t="s">
+        <v>39</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>63</v>
+        <v>52</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H13" s="1"/>
     </row>
@@ -1423,23 +1298,23 @@
       <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>56</v>
-      </c>
       <c r="F14" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>65</v>
+        <v>57</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H14" s="1"/>
     </row>
@@ -1447,23 +1322,23 @@
       <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="9" t="s">
-        <v>50</v>
+      <c r="B15" s="8" t="s">
+        <v>43</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>56</v>
+        <v>44</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>49</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>65</v>
+        <v>57</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H15" s="1"/>
     </row>
@@ -1471,27 +1346,27 @@
       <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>54</v>
+      <c r="B16" s="8" t="s">
+        <v>47</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>56</v>
+        <v>51</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>49</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>65</v>
+        <v>57</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1500,8 +1375,9 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I17" s="1"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1510,46 +1386,52 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I18" s="1"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I19" s="2"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I20" s="2"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I21" s="2"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I22" s="2"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixes typos in excel sheet
</commit_message>
<xml_diff>
--- a/data/Prompt Evaluation.xlsx
+++ b/data/Prompt Evaluation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/merlindconstanzepohl/Desktop/RAG Implementierung/Code/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B2FCE2-A494-7A4B-BC8F-E4B5A1E29FF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C45CD2D-7DB5-6443-9B05-5B6C93531217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1040" yWindow="680" windowWidth="27620" windowHeight="16080" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
+    <workbookView xWindow="160" yWindow="840" windowWidth="28380" windowHeight="15900" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -179,7 +179,363 @@
     </r>
   </si>
   <si>
-    <t>substantial eco-system change and decline: more
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>partially relevant (1)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+correct, but not full information</t>
+    </r>
+  </si>
+  <si>
+    <t>Total reef visits increased from 1.4 million in 1993-94 to just under 2 million visits in 2004-05.(p. 23)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>value provided in documents (1)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>What does happen to the fish if the reef gets in a bad condition?</t>
+  </si>
+  <si>
+    <t>The fish and other organisms dependent on the living coral also die (if they cannot move elsewhere). In turn, the fish and other animals higher up the food chain (including the top predators) also either die or move elsewhere.</t>
+  </si>
+  <si>
+    <t>The text does not mention what happens to the octopus. It only discusses the effects of climate change on coral reefs and the organisms that depend on them, including fish and other animals higher up the food chain.</t>
+  </si>
+  <si>
+    <t>What happens to the octopus?</t>
+  </si>
+  <si>
+    <t>Where is Nemo?</t>
+  </si>
+  <si>
+    <t>There is no mention of Nemo in the provided context.</t>
+  </si>
+  <si>
+    <t>not int the document</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not in the document </t>
+  </si>
+  <si>
+    <t>Can we calculate the total population of Australia?</t>
+  </si>
+  <si>
+    <t>value provided in documents (1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value not provided in documents (1)
+</t>
+  </si>
+  <si>
+    <t>No, the provided context does not mention the total population of Australia. It only provides information on the economic value and employment figures for the Great Barrier Reef Marine Park (GBRMP) in Queensland and Australia.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Correctness
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Retrieval output versus expected text/ground truth</t>
+    </r>
+  </si>
+  <si>
+    <t>not correct</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>relevant (1)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>correct</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Answer Relevancy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Is the answer actually useful for the user’s query?
+Is the output on-topic and addresses the user’s intent?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Faithfulness / Groundedness</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Does the answer come only from the provided documents? 
+Is the response supported by the context?
+Does the model hallucinate?
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Evaluation metrics:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Faithfulness/ Groundedness: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+relevant (1) / partially relevant (1 or 0) / not relevant (0);
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Answer Relevancy: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+value provided in documents / value not provided in documents
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Correctness:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> correct / not correct
+</t>
+    </r>
+  </si>
+  <si>
+    <t>ECO-SYSTEM IMPACTS: [...] The fish and other organisms dependent on the
+living coral also die (if they cannot move elsewhere). In turn, the fish and other animals
+higher up the food chain (including the top predators) also either die or move elsewhere. (p. 57/58)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>partially relevant (0)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+it provides literally the same text, but without the context before it seems a bit abstract and is not well readable fo the user
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>partially relevant (0)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+no hallucination/not wrong, still value not correctly given and answer not properly answered as user clearly asked for a future scenario
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>partially relevant (1)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+no hallucination, still incorrect value because of wrong context -  but seems to be reasonable value to user
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Substantial eco-system change and decline: more
 extreme weather, plus more tropical disease risks, 
 coral bleaching: Reef
 destruction, less coral cover, less biodiversity (p. 5)
@@ -188,363 +544,7 @@
 towards lower species diversity and numbers;
 towards less coral cover;
 towards more specialisation on more hardy coral species;
-and including higher algae concentrations. (58)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>partially relevant (1)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-correct, but not full information</t>
-    </r>
-  </si>
-  <si>
-    <t>Total reef visits increased from 1.4 million in 1993-94 to just under 2 million visits in 2004-05.(p. 23)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>value provided in documents (1)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <t>What does happen to the fish if the reef gets in a bad condition?</t>
-  </si>
-  <si>
-    <t>The fish and other organisms dependent on the living coral also die (if they cannot move elsewhere). In turn, the fish and other animals higher up the food chain (including the top predators) also either die or move elsewhere.</t>
-  </si>
-  <si>
-    <t>The text does not mention what happens to the octopus. It only discusses the effects of climate change on coral reefs and the organisms that depend on them, including fish and other animals higher up the food chain.</t>
-  </si>
-  <si>
-    <t>What happens to the octopus?</t>
-  </si>
-  <si>
-    <t>Where is Nemo?</t>
-  </si>
-  <si>
-    <t>There is no mention of Nemo in the provided context.</t>
-  </si>
-  <si>
-    <t>not int the document</t>
-  </si>
-  <si>
-    <t xml:space="preserve">not in the document </t>
-  </si>
-  <si>
-    <t>Can we calculate the total population of Australia?</t>
-  </si>
-  <si>
-    <t>value provided in documents (1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value not provided in documents (1)
-</t>
-  </si>
-  <si>
-    <t>ECO-SYSTEM IMPACTS: The fish and other organisms dependent on the
-living coral also die (if they cannot move elsewhere). In turn, the fish and other animals
-higher up the food chain (including the top predators) also either die or move elsewhere. (p. 57/58)</t>
-  </si>
-  <si>
-    <t>No, the provided context does not mention the total population of Australia. It only provides information on the economic value and employment figures for the Great Barrier Reef Marine Park (GBRMP) in Queensland and Australia.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>partially relevant (0)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-it provides literally the same text, without the context before it seems a bit abstract and is not well readable
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>partially relevant (1)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-no hallucination/not wrong, still incorrect value because of wrong context -  but could be correct if user doesn't know
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>partially relevant (0)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-no hallucination/not wrong, still value not correctly given and answer not properly answered
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Correctness
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Retrieval output versus expected text/ground truth</t>
-    </r>
-  </si>
-  <si>
-    <t>not correct</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>relevant (1)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <t>correct</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Answer Relevancy</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Is the answer actually useful for the user’s query?
-Is the output on-topic and addresses the user’s intent?
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Faithfulness / Groundedness</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Does the answer come only from the provided documents? 
-Is the response supported by the context?
-Does the model hallucinate?
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Evaluation metrics:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Faithfulness/ Groundedness: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-relevant (1) / partially relevant (1 or 0) / not relevant (0);
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Answer Relevancy: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-value provided in documents / value not provided in documents
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Correctness:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> correct / not correct
-</t>
-    </r>
+and including higher algae concentrations. (p. 58)</t>
   </si>
 </sst>
 </file>
@@ -573,7 +573,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -583,6 +583,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEAF8DB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE1ECF9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -599,7 +605,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -628,6 +634,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -636,6 +645,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFE1ECF9"/>
       <color rgb="FFEAF8DB"/>
     </mruColors>
   </colors>
@@ -994,16 +1004,16 @@
         <v>34</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="68" x14ac:dyDescent="0.2">
@@ -1020,13 +1030,13 @@
         <v>19</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H2" s="1"/>
     </row>
@@ -1044,13 +1054,13 @@
         <v>20</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H3" s="1"/>
     </row>
@@ -1068,13 +1078,13 @@
         <v>21</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H4" s="1"/>
     </row>
@@ -1092,13 +1102,13 @@
         <v>23</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H5" s="1"/>
     </row>
@@ -1110,19 +1120,19 @@
         <v>2</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>24</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H6" s="1"/>
     </row>
@@ -1140,13 +1150,13 @@
         <v>25</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H7" s="1"/>
     </row>
@@ -1164,13 +1174,13 @@
         <v>26</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H8" s="1"/>
     </row>
@@ -1188,17 +1198,17 @@
         <v>27</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H9" s="1"/>
     </row>
-    <row r="10" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1212,13 +1222,13 @@
         <v>28</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H10" s="1"/>
     </row>
@@ -1236,13 +1246,13 @@
         <v>29</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H11" s="1"/>
     </row>
@@ -1254,19 +1264,19 @@
         <v>10</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>30</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H12" s="1"/>
     </row>
@@ -1275,22 +1285,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="E13" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H13" s="1"/>
     </row>
@@ -1299,22 +1309,22 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H14" s="1"/>
     </row>
@@ -1323,22 +1333,22 @@
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>44</v>
-      </c>
       <c r="E15" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H15" s="1"/>
     </row>
@@ -1347,22 +1357,22 @@
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H16" s="1"/>
     </row>

</xml_diff>

<commit_message>
adjustments to the excel table
</commit_message>
<xml_diff>
--- a/data/Prompt Evaluation.xlsx
+++ b/data/Prompt Evaluation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/merlindconstanzepohl/Desktop/RAG Implementierung/Code/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C45CD2D-7DB5-6443-9B05-5B6C93531217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E70065D-858F-E24C-9712-F04F94930644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="840" windowWidth="28380" windowHeight="15900" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
+    <workbookView xWindow="160" yWindow="680" windowWidth="17780" windowHeight="16060" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="69">
   <si>
     <t>Query</t>
   </si>
@@ -546,12 +546,33 @@
 towards more specialisation on more hardy coral species;
 and including higher algae concentrations. (p. 58)</t>
   </si>
+  <si>
+    <t>Top-k</t>
+  </si>
+  <si>
+    <t>Found relevant chunks</t>
+  </si>
+  <si>
+    <t>Relevant chunks in source</t>
+  </si>
+  <si>
+    <t>Precision@k</t>
+  </si>
+  <si>
+    <t>Recall@k</t>
+  </si>
+  <si>
+    <t>Hit Rate</t>
+  </si>
+  <si>
+    <t>F1@5</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -569,6 +590,13 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
@@ -605,7 +633,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -636,6 +664,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -977,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{483B6C7E-3945-004D-9C20-B4D0D386A596}">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -985,12 +1016,17 @@
     <col min="3" max="4" width="42.1640625" customWidth="1"/>
     <col min="5" max="5" width="42.1640625" style="2" customWidth="1"/>
     <col min="6" max="7" width="53.6640625" customWidth="1"/>
-    <col min="8" max="8" width="39.1640625" customWidth="1"/>
-    <col min="9" max="9" width="40.83203125" customWidth="1"/>
-    <col min="10" max="10" width="42" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" customWidth="1"/>
+    <col min="9" max="9" width="22.33203125" customWidth="1"/>
+    <col min="10" max="10" width="25.5" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" customWidth="1"/>
+    <col min="12" max="14" width="13.33203125" customWidth="1"/>
+    <col min="15" max="15" width="39.1640625" customWidth="1"/>
+    <col min="16" max="16" width="40.83203125" customWidth="1"/>
+    <col min="17" max="17" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="155" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" ht="155" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>12</v>
       </c>
@@ -1012,11 +1048,32 @@
       <c r="G1" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="O1" s="10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" ht="68" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1038,9 +1095,21 @@
       <c r="G2" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="H2" s="1"/>
-    </row>
-    <row r="3" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="H2" s="11">
+        <v>5</v>
+      </c>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" t="e">
+        <f>2 * (B2 * C2) / (B2 + C2)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O2" s="1"/>
+    </row>
+    <row r="3" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1062,9 +1131,18 @@
       <c r="G3" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="H3" s="11">
+        <v>5</v>
+      </c>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="1"/>
+    </row>
+    <row r="4" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1086,9 +1164,18 @@
       <c r="G4" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H4" s="1"/>
-    </row>
-    <row r="5" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="H4" s="11">
+        <v>5</v>
+      </c>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="1"/>
+    </row>
+    <row r="5" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1110,9 +1197,18 @@
       <c r="G5" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H5" s="1"/>
-    </row>
-    <row r="6" spans="1:8" ht="238" x14ac:dyDescent="0.2">
+      <c r="H5" s="11">
+        <v>5</v>
+      </c>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="1"/>
+    </row>
+    <row r="6" spans="1:15" ht="238" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1134,9 +1230,18 @@
       <c r="G6" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H6" s="1"/>
-    </row>
-    <row r="7" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+      <c r="H6" s="11">
+        <v>5</v>
+      </c>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="1:15" ht="119" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1158,9 +1263,18 @@
       <c r="G7" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H7" s="1"/>
-    </row>
-    <row r="8" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="H7" s="11">
+        <v>5</v>
+      </c>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="1"/>
+    </row>
+    <row r="8" spans="1:15" ht="68" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1182,9 +1296,18 @@
       <c r="G8" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H8" s="1"/>
-    </row>
-    <row r="9" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="H8" s="11">
+        <v>5</v>
+      </c>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="1"/>
+    </row>
+    <row r="9" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1206,9 +1329,18 @@
       <c r="G9" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H9" s="1"/>
-    </row>
-    <row r="10" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="H9" s="11">
+        <v>5</v>
+      </c>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="1"/>
+    </row>
+    <row r="10" spans="1:15" ht="85" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1230,9 +1362,18 @@
       <c r="G10" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="H10" s="1"/>
-    </row>
-    <row r="11" spans="1:8" ht="170" x14ac:dyDescent="0.2">
+      <c r="H10" s="11">
+        <v>5</v>
+      </c>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="1"/>
+    </row>
+    <row r="11" spans="1:15" ht="170" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1254,9 +1395,18 @@
       <c r="G11" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H11" s="1"/>
-    </row>
-    <row r="12" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="H11" s="11">
+        <v>5</v>
+      </c>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="1"/>
+    </row>
+    <row r="12" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1278,9 +1428,18 @@
       <c r="G12" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H12" s="1"/>
-    </row>
-    <row r="13" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+      <c r="H12" s="11">
+        <v>5</v>
+      </c>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="1"/>
+    </row>
+    <row r="13" spans="1:15" ht="119" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1302,9 +1461,18 @@
       <c r="G13" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H13" s="1"/>
-    </row>
-    <row r="14" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="H13" s="11">
+        <v>5</v>
+      </c>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="1"/>
+    </row>
+    <row r="14" spans="1:15" ht="85" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1326,9 +1494,18 @@
       <c r="G14" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H14" s="1"/>
-    </row>
-    <row r="15" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="H14" s="11">
+        <v>5</v>
+      </c>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="1"/>
+    </row>
+    <row r="15" spans="1:15" ht="34" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1350,9 +1527,18 @@
       <c r="G15" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H15" s="1"/>
-    </row>
-    <row r="16" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+      <c r="H15" s="11">
+        <v>5</v>
+      </c>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="1"/>
+    </row>
+    <row r="16" spans="1:15" ht="102" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1374,9 +1560,18 @@
       <c r="G16" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H16" s="11">
+        <v>5</v>
+      </c>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="1"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1384,10 +1579,17 @@
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
+      <c r="H17" s="11"/>
       <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1397,8 +1599,15 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -1406,8 +1615,15 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+      <c r="P19" s="2"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -1415,8 +1631,15 @@
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
+      <c r="O20" s="2"/>
+      <c r="P20" s="2"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -1424,8 +1647,15 @@
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
+      <c r="O21" s="2"/>
+      <c r="P21" s="2"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -1433,8 +1663,15 @@
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2"/>
+      <c r="P22" s="2"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -1442,8 +1679,20 @@
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
+      <c r="O23" s="2"/>
+      <c r="P23" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="K1" r:id="rId1" xr:uid="{8245B373-7B93-6F42-BD9E-41C920E87C6E}"/>
+    <hyperlink ref="L1" r:id="rId2" xr:uid="{91FC8E1C-8310-2A41-BD46-A995EE8D0058}"/>
+    <hyperlink ref="N1" r:id="rId3" xr:uid="{79158C6D-8DE3-3143-A72D-1A10BCFA2C44}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>